<commit_message>
Record 17:11 live forecasts and settle seven confirmed prior forecasts
</commit_message>
<xml_diff>
--- a/Live ТБ/Live ТБ.xlsx
+++ b/Live ТБ/Live ТБ.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="1" r:id="R97522867614449da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр" sheetId="2" r:id="Rb8619bd57ec84073"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Правила" sheetId="3" r:id="R68faba8d7cde4584"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="1" r:id="R518d3d0de3904d0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр" sheetId="2" r:id="Rb8b4f380b534441c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Правила" sheetId="3" r:id="R3d7c7b229e7d42c1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -889,11 +889,11 @@
       </x:c>
       <x:c r="C6" s="124" t="n">
         <x:f>COUNTIFS('Реестр'!$Y$6:$Y$505,"Оптимальный")</x:f>
-        <x:v>7</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D6" s="124" t="n">
         <x:f>COUNTIFS('Реестр'!$Y$6:$Y$505,"Агрессивный")</x:f>
-        <x:v>7</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E6"/>
       <x:c r="F6"/>
@@ -910,11 +910,11 @@
       </x:c>
       <x:c r="C7" s="124" t="n">
         <x:f>COUNTIFS('Реестр'!$Y$6:$Y$505,"Оптимальный",'Реестр'!$W$6:$W$505,"Рассчитан")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D7" s="124" t="n">
         <x:f>COUNTIFS('Реестр'!$Y$6:$Y$505,"Агрессивный",'Реестр'!$W$6:$W$505,"Рассчитан")</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E7"/>
       <x:c r="F7"/>
@@ -935,7 +935,7 @@
       </x:c>
       <x:c r="D8" s="124" t="n">
         <x:f>COUNTIFS('Реестр'!$Y$6:$Y$505,"Агрессивный",'Реестр'!$W$6:$W$505,"Открыт")</x:f>
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E8"/>
       <x:c r="F8"/>
@@ -952,7 +952,7 @@
       </x:c>
       <x:c r="C9" s="124" t="n">
         <x:f>COUNTIFS('Реестр'!$Y$6:$Y$505,"Оптимальный",'Реестр'!$U$6:$U$505,"Выигрыш")+COUNTIFS('Реестр'!$Y$6:$Y$505,"Оптимальный",'Реестр'!$U$6:$U$505,"Плюс")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="124" t="n">
         <x:f>COUNTIFS('Реестр'!$Y$6:$Y$505,"Агрессивный",'Реестр'!$U$6:$U$505,"Выигрыш")+COUNTIFS('Реестр'!$Y$6:$Y$505,"Агрессивный",'Реестр'!$U$6:$U$505,"Плюс")</x:f>
@@ -998,7 +998,7 @@
       </x:c>
       <x:c r="D11" s="124" t="n">
         <x:f>COUNTIFS('Реестр'!$Y$6:$Y$505,"Агрессивный",'Реестр'!$U$6:$U$505,"Возврат")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E11"/>
       <x:c r="F11"/>
@@ -1036,11 +1036,11 @@
       </x:c>
       <x:c r="C13" s="124" t="n">
         <x:f>COUNTIFS('Реестр'!$Y$6:$Y$505,"Оптимальный",'Реестр'!$U$6:$U$505,"Поражение")+COUNTIFS('Реестр'!$Y$6:$Y$505,"Оптимальный",'Реестр'!$U$6:$U$505,"Минус")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D13" s="124" t="n">
         <x:f>COUNTIFS('Реестр'!$Y$6:$Y$505,"Агрессивный",'Реестр'!$U$6:$U$505,"Поражение")+COUNTIFS('Реестр'!$Y$6:$Y$505,"Агрессивный",'Реестр'!$U$6:$U$505,"Минус")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E13"/>
       <x:c r="F13"/>
@@ -1057,11 +1057,11 @@
       </x:c>
       <x:c r="C14" s="128" t="n">
         <x:f>SUMIFS('Реестр'!$V$6:$V$505,'Реестр'!$Y$6:$Y$505,"Оптимальный",'Реестр'!$W$6:$W$505,"Рассчитан")</x:f>
-        <x:v>0</x:v>
+        <x:v>-1.4</x:v>
       </x:c>
       <x:c r="D14" s="128" t="n">
         <x:f>SUMIFS('Реестр'!$V$6:$V$505,'Реестр'!$Y$6:$Y$505,"Агрессивный",'Реестр'!$W$6:$W$505,"Рассчитан")</x:f>
-        <x:v>0</x:v>
+        <x:v>-3</x:v>
       </x:c>
       <x:c r="E14"/>
       <x:c r="F14"/>
@@ -1076,11 +1076,13 @@
         <x:f>IF(B7=0,"",B14/B7)</x:f>
         <x:v>0.06981132075471698</x:v>
       </x:c>
-      <x:c r="C15" s="129" t="str">
+      <x:c r="C15" s="129" t="n">
         <x:f>IF(C7=0,"",C14/C7)</x:f>
-      </x:c>
-      <x:c r="D15" s="129" t="str">
+        <x:v>-0.4666666666666666</x:v>
+      </x:c>
+      <x:c r="D15" s="129" t="n">
         <x:f>IF(D7=0,"",D14/D7)</x:f>
+        <x:v>-0.75</x:v>
       </x:c>
       <x:c r="E15"/>
       <x:c r="F15"/>
@@ -1095,11 +1097,13 @@
         <x:f>IF(B7=0,"",SUMIFS('Реестр'!$J$6:$J$505,'Реестр'!$Y$6:$Y$505,"История без разделения",'Реестр'!$W$6:$W$505,"Рассчитан")/B7)</x:f>
         <x:v>1.9047169811320754</x:v>
       </x:c>
-      <x:c r="C16" s="125" t="str">
+      <x:c r="C16" s="125" t="n">
         <x:f>IF(C7=0,"",SUMIFS('Реестр'!$J$6:$J$505,'Реестр'!$Y$6:$Y$505,"Оптимальный",'Реестр'!$W$6:$W$505,"Рассчитан")/C7)</x:f>
-      </x:c>
-      <x:c r="D16" s="125" t="str">
+        <x:v>1.5527666666666669</x:v>
+      </x:c>
+      <x:c r="D16" s="125" t="n">
         <x:f>IF(D7=0,"",SUMIFS('Реестр'!$J$6:$J$505,'Реестр'!$Y$6:$Y$505,"Агрессивный",'Реестр'!$W$6:$W$505,"Рассчитан")/D7)</x:f>
+        <x:v>2.0625</x:v>
       </x:c>
       <x:c r="E16"/>
       <x:c r="F16"/>
@@ -1114,11 +1118,13 @@
         <x:f>IF(B7=0,"",(B9+B10)/B7)</x:f>
         <x:v>0.5283018867924528</x:v>
       </x:c>
-      <x:c r="C17" s="126" t="str">
+      <x:c r="C17" s="126" t="n">
         <x:f>IF(C7=0,"",(C9+C10)/C7)</x:f>
-      </x:c>
-      <x:c r="D17" s="126" t="str">
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="D17" s="126" t="n">
         <x:f>IF(D7=0,"",(D9+D10)/D7)</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
@@ -1142,11 +1148,11 @@
       <x:c r="B20" s="124"/>
       <x:c r="C20" s="124" t="n">
         <x:f>COUNTIFS('Реестр'!$Y$6:$Y$505,"Оптимальный",'Реестр'!$AE$6:$AE$505,"Да")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D20" s="124" t="n">
         <x:f>COUNTIFS('Реестр'!$Y$6:$Y$505,"Агрессивный",'Реестр'!$AE$6:$AE$505,"Да")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="23" customHeight="1">
@@ -1156,11 +1162,11 @@
       <x:c r="B21" s="128"/>
       <x:c r="C21" s="128" t="n">
         <x:f>SUMIFS('Реестр'!$V$6:$V$505,'Реестр'!$Y$6:$Y$505,"Оптимальный",'Реестр'!$AE$6:$AE$505,"Да")</x:f>
-        <x:v>0</x:v>
+        <x:v>-1.4</x:v>
       </x:c>
       <x:c r="D21" s="128" t="n">
         <x:f>SUMIFS('Реестр'!$V$6:$V$505,'Реестр'!$Y$6:$Y$505,"Агрессивный",'Реестр'!$AE$6:$AE$505,"Да")</x:f>
-        <x:v>0</x:v>
+        <x:v>-2</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
@@ -1168,11 +1174,13 @@
         <x:v>ROI по парам</x:v>
       </x:c>
       <x:c r="B22" s="129"/>
-      <x:c r="C22" s="129" t="str">
+      <x:c r="C22" s="129" t="n">
         <x:f>IF(C20=0,"",C21/C20)</x:f>
-      </x:c>
-      <x:c r="D22" s="129" t="str">
+        <x:v>-0.4666666666666666</x:v>
+      </x:c>
+      <x:c r="D22" s="129" t="n">
         <x:f>IF(D20=0,"",D21/D20)</x:f>
+        <x:v>-0.6666666666666666</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
@@ -1180,11 +1188,13 @@
         <x:v>Средний коэф. по парам</x:v>
       </x:c>
       <x:c r="B23" s="125"/>
-      <x:c r="C23" s="125" t="str">
+      <x:c r="C23" s="125" t="n">
         <x:f>IF(C20=0,"",SUMIFS('Реестр'!$J$6:$J$505,'Реестр'!$Y$6:$Y$505,"Оптимальный",'Реестр'!$AE$6:$AE$505,"Да")/C20)</x:f>
-      </x:c>
-      <x:c r="D23" s="125" t="str">
+        <x:v>1.5527666666666669</x:v>
+      </x:c>
+      <x:c r="D23" s="125" t="n">
         <x:f>IF(D20=0,"",SUMIFS('Реестр'!$J$6:$J$505,'Реестр'!$Y$6:$Y$505,"Агрессивный",'Реестр'!$AE$6:$AE$505,"Да")/D20)</x:f>
+        <x:v>2.058333333333333</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -6349,14 +6359,19 @@
       <x:c r="S59" s="80" t="str">
         <x:v>BetsAPI / Bet365 full markets; Резервная команда против взрослой; run 38538525336 attempt 2</x:v>
       </x:c>
-      <x:c r="T59" s="80"/>
-      <x:c r="U59" s="80"/>
-      <x:c r="V59" s="89" t="str">
+      <x:c r="T59" s="80" t="str">
+        <x:v>0:1</x:v>
+      </x:c>
+      <x:c r="U59" s="80" t="str">
+        <x:v>Поражение</x:v>
+      </x:c>
+      <x:c r="V59" s="89" t="n">
         <x:f>IF(A59="","",IF(U59="","",IF(U59="Выигрыш",J59-1,IF(U59="Полувыигрыш",(J59-1)/2,IF(U59="Возврат",0,IF(U59="Полупроигрыш",-0.5,IF(U59="Поражение",-1,"Проверить результат")))))))</x:f>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="W59" s="80" t="str">
         <x:f>IF(A59="","",IF(U59="","Открыт",IF(ISNUMBER(V59),"Рассчитан","Проверить результат")))</x:f>
-        <x:v>Открыт</x:v>
+        <x:v>Рассчитан</x:v>
       </x:c>
       <x:c r="X59" s="98" t="str">
         <x:v>Ещё 1 гол - возврат; исходные условия первичного ответа</x:v>
@@ -6381,9 +6396,11 @@
       </x:c>
       <x:c r="AE59" s="5" t="str">
         <x:f>IF(A59="","",IF(Z59="","Нет ID пары",IF(AND(COUNTIFS($Z$59:$Z$505,Z59,$Y$59:$Y$505,"Оптимальный",$W$59:$W$505,"Рассчитан")=1,COUNTIFS($Z$59:$Z$505,Z59,$Y$59:$Y$505,"Агрессивный",$W$59:$W$505,"Рассчитан")=1),"Да","Нет")))</x:f>
-        <x:v>Нет</x:v>
-      </x:c>
-      <x:c r="AF59" s="5"/>
+        <x:v>Да</x:v>
+      </x:c>
+      <x:c r="AF59" s="5" t="str">
+        <x:v>https://www.sofascore.com/football/match/olympiacos-athens-kallithea-fc/fpbsFoid | FT 0:1; матч завершён | Проверено 14.10.2026 17:14:56 МСК</x:v>
+      </x:c>
       <x:c r="AG59" s="5" t="str">
         <x:v>Два контура v2</x:v>
       </x:c>
@@ -6446,14 +6463,19 @@
       <x:c r="S60" s="80" t="str">
         <x:v>BetsAPI / Bet365 full markets; Резервная команда против взрослой; run 38538525336 attempt 2</x:v>
       </x:c>
-      <x:c r="T60" s="80"/>
-      <x:c r="U60" s="80"/>
-      <x:c r="V60" s="89" t="str">
+      <x:c r="T60" s="80" t="str">
+        <x:v>0:1</x:v>
+      </x:c>
+      <x:c r="U60" s="80" t="str">
+        <x:v>Поражение</x:v>
+      </x:c>
+      <x:c r="V60" s="89" t="n">
         <x:f>IF(A60="","",IF(U60="","",IF(U60="Выигрыш",J60-1,IF(U60="Полувыигрыш",(J60-1)/2,IF(U60="Возврат",0,IF(U60="Полупроигрыш",-0.5,IF(U60="Поражение",-1,"Проверить результат")))))))</x:f>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="W60" s="80" t="str">
         <x:f>IF(A60="","",IF(U60="","Открыт",IF(ISNUMBER(V60),"Рассчитан","Проверить результат")))</x:f>
-        <x:v>Открыт</x:v>
+        <x:v>Рассчитан</x:v>
       </x:c>
       <x:c r="X60" s="98" t="str">
         <x:v>Без возврата; исходные условия первичного ответа</x:v>
@@ -6478,9 +6500,11 @@
       </x:c>
       <x:c r="AE60" s="5" t="str">
         <x:f>IF(A60="","",IF(Z60="","Нет ID пары",IF(AND(COUNTIFS($Z$59:$Z$505,Z60,$Y$59:$Y$505,"Оптимальный",$W$59:$W$505,"Рассчитан")=1,COUNTIFS($Z$59:$Z$505,Z60,$Y$59:$Y$505,"Агрессивный",$W$59:$W$505,"Рассчитан")=1),"Да","Нет")))</x:f>
-        <x:v>Нет</x:v>
-      </x:c>
-      <x:c r="AF60" s="5"/>
+        <x:v>Да</x:v>
+      </x:c>
+      <x:c r="AF60" s="5" t="str">
+        <x:v>https://www.sofascore.com/football/match/olympiacos-athens-kallithea-fc/fpbsFoid | FT 0:1; матч завершён | Проверено 14.10.2026 17:14:56 МСК</x:v>
+      </x:c>
       <x:c r="AG60" s="5" t="str">
         <x:v>Два контура v2</x:v>
       </x:c>
@@ -6543,14 +6567,19 @@
       <x:c r="S61" s="80" t="str">
         <x:v>BetsAPI / Bet365 full markets; Молодёжный/юниорский; run 38538525336 attempt 2</x:v>
       </x:c>
-      <x:c r="T61" s="80"/>
-      <x:c r="U61" s="80"/>
-      <x:c r="V61" s="89" t="str">
+      <x:c r="T61" s="80" t="str">
+        <x:v>4:0</x:v>
+      </x:c>
+      <x:c r="U61" s="80" t="str">
+        <x:v>Выигрыш</x:v>
+      </x:c>
+      <x:c r="V61" s="89" t="n">
         <x:f>IF(A61="","",IF(U61="","",IF(U61="Выигрыш",J61-1,IF(U61="Полувыигрыш",(J61-1)/2,IF(U61="Возврат",0,IF(U61="Полупроигрыш",-0.5,IF(U61="Поражение",-1,"Проверить результат")))))))</x:f>
+        <x:v>0.6000000000000001</x:v>
       </x:c>
       <x:c r="W61" s="80" t="str">
         <x:f>IF(A61="","",IF(U61="","Открыт",IF(ISNUMBER(V61),"Рассчитан","Проверить результат")))</x:f>
-        <x:v>Открыт</x:v>
+        <x:v>Рассчитан</x:v>
       </x:c>
       <x:c r="X61" s="98" t="str">
         <x:v>Без возврата; исходные условия первичного ответа</x:v>
@@ -6575,9 +6604,11 @@
       </x:c>
       <x:c r="AE61" s="5" t="str">
         <x:f>IF(A61="","",IF(Z61="","Нет ID пары",IF(AND(COUNTIFS($Z$59:$Z$505,Z61,$Y$59:$Y$505,"Оптимальный",$W$59:$W$505,"Рассчитан")=1,COUNTIFS($Z$59:$Z$505,Z61,$Y$59:$Y$505,"Агрессивный",$W$59:$W$505,"Рассчитан")=1),"Да","Нет")))</x:f>
-        <x:v>Нет</x:v>
-      </x:c>
-      <x:c r="AF61" s="5"/>
+        <x:v>Да</x:v>
+      </x:c>
+      <x:c r="AF61" s="5" t="str">
+        <x:v>https://www.sofascore.com/football/match/partizani-tirana-u19-u19-valletta-u19/AQRgsxFik | FT 4:0; матч завершён; суммарный счёт двух матчей 6:0 не используется | Проверено 14.10.2026 17:14:56 МСК</x:v>
+      </x:c>
       <x:c r="AG61" s="5" t="str">
         <x:v>Два контура v2</x:v>
       </x:c>
@@ -6640,14 +6671,19 @@
       <x:c r="S62" s="80" t="str">
         <x:v>BetsAPI / Bet365 full markets; Молодёжный/юниорский; run 38538525336 attempt 2</x:v>
       </x:c>
-      <x:c r="T62" s="80"/>
-      <x:c r="U62" s="80"/>
-      <x:c r="V62" s="89" t="str">
+      <x:c r="T62" s="80" t="str">
+        <x:v>4:0</x:v>
+      </x:c>
+      <x:c r="U62" s="80" t="str">
+        <x:v>Возврат</x:v>
+      </x:c>
+      <x:c r="V62" s="89" t="n">
         <x:f>IF(A62="","",IF(U62="","",IF(U62="Выигрыш",J62-1,IF(U62="Полувыигрыш",(J62-1)/2,IF(U62="Возврат",0,IF(U62="Полупроигрыш",-0.5,IF(U62="Поражение",-1,"Проверить результат")))))))</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="W62" s="80" t="str">
         <x:f>IF(A62="","",IF(U62="","Открыт",IF(ISNUMBER(V62),"Рассчитан","Проверить результат")))</x:f>
-        <x:v>Открыт</x:v>
+        <x:v>Рассчитан</x:v>
       </x:c>
       <x:c r="X62" s="98" t="str">
         <x:v>Ещё 2 гола - возврат; исходные условия первичного ответа</x:v>
@@ -6672,9 +6708,11 @@
       </x:c>
       <x:c r="AE62" s="5" t="str">
         <x:f>IF(A62="","",IF(Z62="","Нет ID пары",IF(AND(COUNTIFS($Z$59:$Z$505,Z62,$Y$59:$Y$505,"Оптимальный",$W$59:$W$505,"Рассчитан")=1,COUNTIFS($Z$59:$Z$505,Z62,$Y$59:$Y$505,"Агрессивный",$W$59:$W$505,"Рассчитан")=1),"Да","Нет")))</x:f>
-        <x:v>Нет</x:v>
-      </x:c>
-      <x:c r="AF62" s="5"/>
+        <x:v>Да</x:v>
+      </x:c>
+      <x:c r="AF62" s="5" t="str">
+        <x:v>https://www.sofascore.com/football/match/partizani-tirana-u19-u19-valletta-u19/AQRgsxFik | FT 4:0; матч завершён; ТБ 4 возвращён | Проверено 14.10.2026 17:14:56 МСК</x:v>
+      </x:c>
       <x:c r="AG62" s="5" t="str">
         <x:v>Два контура v2</x:v>
       </x:c>
@@ -6834,14 +6872,19 @@
       <x:c r="S64" s="80" t="str">
         <x:v>BetsAPI / Bet365 full markets; Взрослый мужской; run 38538525336 attempt 2</x:v>
       </x:c>
-      <x:c r="T64" s="80"/>
-      <x:c r="U64" s="80"/>
-      <x:c r="V64" s="89" t="str">
+      <x:c r="T64" s="80" t="str">
+        <x:v>1:1</x:v>
+      </x:c>
+      <x:c r="U64" s="80" t="str">
+        <x:v>Поражение</x:v>
+      </x:c>
+      <x:c r="V64" s="89" t="n">
         <x:f>IF(A64="","",IF(U64="","",IF(U64="Выигрыш",J64-1,IF(U64="Полувыигрыш",(J64-1)/2,IF(U64="Возврат",0,IF(U64="Полупроигрыш",-0.5,IF(U64="Поражение",-1,"Проверить результат")))))))</x:f>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="W64" s="80" t="str">
         <x:f>IF(A64="","",IF(U64="","Открыт",IF(ISNUMBER(V64),"Рассчитан","Проверить результат")))</x:f>
-        <x:v>Открыт</x:v>
+        <x:v>Рассчитан</x:v>
       </x:c>
       <x:c r="X64" s="98" t="str">
         <x:v>Гол до перерыва; исходные условия первичного ответа</x:v>
@@ -6868,7 +6911,9 @@
         <x:f>IF(A64="","",IF(Z64="","Нет ID пары",IF(AND(COUNTIFS($Z$59:$Z$505,Z64,$Y$59:$Y$505,"Оптимальный",$W$59:$W$505,"Рассчитан")=1,COUNTIFS($Z$59:$Z$505,Z64,$Y$59:$Y$505,"Агрессивный",$W$59:$W$505,"Рассчитан")=1),"Да","Нет")))</x:f>
         <x:v>Нет</x:v>
       </x:c>
-      <x:c r="AF64" s="5"/>
+      <x:c r="AF64" s="5" t="str">
+        <x:v>https://www.sofascore.com/football/match/sporting-alexandria-alexandria-petroleum/AWcesKjie | HT 1:1; первый тайм завершён | Проверено 14.10.2026 17:14:56 МСК</x:v>
+      </x:c>
       <x:c r="AG64" s="5" t="str">
         <x:v>Два контура v2</x:v>
       </x:c>
@@ -6931,14 +6976,19 @@
       <x:c r="S65" s="80" t="str">
         <x:v>BetsAPI / Bet365 full markets; Взрослый мужской; run 38538525336 attempt 2</x:v>
       </x:c>
-      <x:c r="T65" s="80"/>
-      <x:c r="U65" s="80"/>
-      <x:c r="V65" s="89" t="str">
+      <x:c r="T65" s="80" t="str">
+        <x:v>0:0</x:v>
+      </x:c>
+      <x:c r="U65" s="80" t="str">
+        <x:v>Поражение</x:v>
+      </x:c>
+      <x:c r="V65" s="89" t="n">
         <x:f>IF(A65="","",IF(U65="","",IF(U65="Выигрыш",J65-1,IF(U65="Полувыигрыш",(J65-1)/2,IF(U65="Возврат",0,IF(U65="Полупроигрыш",-0.5,IF(U65="Поражение",-1,"Проверить результат")))))))</x:f>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="W65" s="80" t="str">
         <x:f>IF(A65="","",IF(U65="","Открыт",IF(ISNUMBER(V65),"Рассчитан","Проверить результат")))</x:f>
-        <x:v>Открыт</x:v>
+        <x:v>Рассчитан</x:v>
       </x:c>
       <x:c r="X65" s="98" t="str">
         <x:v>Гол до перерыва; исходные условия первичного ответа</x:v>
@@ -6963,9 +7013,11 @@
       </x:c>
       <x:c r="AE65" s="5" t="str">
         <x:f>IF(A65="","",IF(Z65="","Нет ID пары",IF(AND(COUNTIFS($Z$59:$Z$505,Z65,$Y$59:$Y$505,"Оптимальный",$W$59:$W$505,"Рассчитан")=1,COUNTIFS($Z$59:$Z$505,Z65,$Y$59:$Y$505,"Агрессивный",$W$59:$W$505,"Рассчитан")=1),"Да","Нет")))</x:f>
-        <x:v>Нет</x:v>
-      </x:c>
-      <x:c r="AF65" s="5"/>
+        <x:v>Да</x:v>
+      </x:c>
+      <x:c r="AF65" s="5" t="str">
+        <x:v>https://www.live-result.com/football/matches/match1800494_TJ_Druzstevnik_Velke_Ludince-Lokomotiva_Zvolen-live-online | Первый тайм 0:0 по статистике периода и хронологии; голы 46 и 76 минут во втором тайме. Согласуется со срезом BetsAPI на перерыве 16:25:03. | Проверено 14.10.2026 17:14:56 МСК</x:v>
+      </x:c>
       <x:c r="AG65" s="5" t="str">
         <x:v>Два контура v2</x:v>
       </x:c>
@@ -7028,14 +7080,19 @@
       <x:c r="S66" s="80" t="str">
         <x:v>BetsAPI / Bet365 full markets; Взрослый мужской; run 38538525336 attempt 2</x:v>
       </x:c>
-      <x:c r="T66" s="80"/>
-      <x:c r="U66" s="80"/>
-      <x:c r="V66" s="89" t="str">
+      <x:c r="T66" s="80" t="str">
+        <x:v>0:0</x:v>
+      </x:c>
+      <x:c r="U66" s="80" t="str">
+        <x:v>Поражение</x:v>
+      </x:c>
+      <x:c r="V66" s="89" t="n">
         <x:f>IF(A66="","",IF(U66="","",IF(U66="Выигрыш",J66-1,IF(U66="Полувыигрыш",(J66-1)/2,IF(U66="Возврат",0,IF(U66="Полупроигрыш",-0.5,IF(U66="Поражение",-1,"Проверить результат")))))))</x:f>
+        <x:v>-1</x:v>
       </x:c>
       <x:c r="W66" s="80" t="str">
         <x:f>IF(A66="","",IF(U66="","Открыт",IF(ISNUMBER(V66),"Рассчитан","Проверить результат")))</x:f>
-        <x:v>Открыт</x:v>
+        <x:v>Рассчитан</x:v>
       </x:c>
       <x:c r="X66" s="98" t="str">
         <x:v>1 гол до перерыва - полувыигрыш; 2 - полный; исходные условия первичного ответа</x:v>
@@ -7060,9 +7117,11 @@
       </x:c>
       <x:c r="AE66" s="5" t="str">
         <x:f>IF(A66="","",IF(Z66="","Нет ID пары",IF(AND(COUNTIFS($Z$59:$Z$505,Z66,$Y$59:$Y$505,"Оптимальный",$W$59:$W$505,"Рассчитан")=1,COUNTIFS($Z$59:$Z$505,Z66,$Y$59:$Y$505,"Агрессивный",$W$59:$W$505,"Рассчитан")=1),"Да","Нет")))</x:f>
-        <x:v>Нет</x:v>
-      </x:c>
-      <x:c r="AF66" s="5"/>
+        <x:v>Да</x:v>
+      </x:c>
+      <x:c r="AF66" s="5" t="str">
+        <x:v>https://www.live-result.com/football/matches/match1800494_TJ_Druzstevnik_Velke_Ludince-Lokomotiva_Zvolen-live-online | Первый тайм 0:0 по статистике периода и хронологии; голы 46 и 76 минут во втором тайме. Согласуется со срезом BetsAPI на перерыве 16:25:03. | Проверено 14.10.2026 17:14:56 МСК</x:v>
+      </x:c>
       <x:c r="AG66" s="5" t="str">
         <x:v>Два контура v2</x:v>
       </x:c>
@@ -7650,25 +7709,63 @@
       </x:c>
     </x:row>
     <x:row r="73">
-      <x:c r="A73" s="80"/>
-      <x:c r="B73" s="80"/>
-      <x:c r="C73" s="83"/>
-      <x:c r="D73" s="80"/>
-      <x:c r="E73" s="80"/>
-      <x:c r="F73" s="86"/>
-      <x:c r="G73" s="80"/>
-      <x:c r="H73" s="95"/>
-      <x:c r="I73" s="95"/>
-      <x:c r="J73" s="96"/>
-      <x:c r="K73" s="97"/>
-      <x:c r="L73" s="98"/>
-      <x:c r="M73" s="98"/>
-      <x:c r="N73" s="98"/>
-      <x:c r="O73" s="98"/>
-      <x:c r="P73" s="98"/>
-      <x:c r="Q73" s="80"/>
-      <x:c r="R73" s="80"/>
-      <x:c r="S73" s="80"/>
+      <x:c r="A73" s="80" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="B73" s="80" t="str">
+        <x:v>11168551</x:v>
+      </x:c>
+      <x:c r="C73" s="83" t="str">
+        <x:v>14.10.2026 17:11:23</x:v>
+      </x:c>
+      <x:c r="D73" s="80" t="str">
+        <x:v>Норвегия — 1-й дивизион</x:v>
+      </x:c>
+      <x:c r="E73" s="80" t="str">
+        <x:v>Стрёммен - Осане</x:v>
+      </x:c>
+      <x:c r="F73" s="86" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="G73" s="80" t="str">
+        <x:v>2:0</x:v>
+      </x:c>
+      <x:c r="H73" s="95" t="str">
+        <x:v>Высокий объём ударов при преимуществе хозяев; возможны голы через давление хозяев и попытки гостей отыграться.</x:v>
+      </x:c>
+      <x:c r="I73" s="95" t="str">
+        <x:v>ТБ 3.25 матча</x:v>
+      </x:c>
+      <x:c r="J73" s="96" t="n">
+        <x:v>1.55</x:v>
+      </x:c>
+      <x:c r="K73" s="97" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L73" s="98" t="str">
+        <x:v>Взрослый мужской. В створ 6:1; мимо 5:9; опасные атаки 50:35; угловые 7:3; xG отсутствует.</x:v>
+      </x:c>
+      <x:c r="M73" s="98" t="str">
+        <x:v>2893.5 с между срезами; минута 22 → 53; с перерывом; не окно 10–15 минут. Прирост в створ 5:1, мимо 4:3, угловые 5:1, опасные атаки 30:25.</x:v>
+      </x:c>
+      <x:c r="N73" s="98" t="str">
+        <x:v>21 удар, в створ 6:1, угловые 7:3. Хозяева способны создавать голы сами, гости отвечают объёмом ударов.</x:v>
+      </x:c>
+      <x:c r="O73" s="98" t="str">
+        <x:v>При 2:0 хозяева могут снижать темп; у гостей лишь 1 удар в створ. Нет xG и короткого интервала динамики.</x:v>
+      </x:c>
+      <x:c r="P73" s="98" t="str">
+        <x:v>Есть счёт, минута, статистика и активные линии; нет xG и динамики за 10–15 минут.</x:v>
+      </x:c>
+      <x:c r="Q73" s="80" t="str">
+        <x:v>ПОДХОДИТ В LIVE</x:v>
+      </x:c>
+      <x:c r="R73" s="80" t="str">
+        <x:v>Канон 14.10.2026; быстрый отбор + сохранение срезов</x:v>
+      </x:c>
+      <x:c r="S73" s="80" t="str">
+        <x:v>BetsAPI Events board + Bet365 full markets; run 38578271681</x:v>
+      </x:c>
       <x:c r="T73" s="80"/>
       <x:c r="U73" s="80"/>
       <x:c r="V73" s="89" t="str">
@@ -7676,40 +7773,96 @@
       </x:c>
       <x:c r="W73" s="80" t="str">
         <x:f>IF(A73="","",IF(U73="","Открыт",IF(ISNUMBER(V73),"Рассчитан","Проверить результат")))</x:f>
-      </x:c>
-      <x:c r="X73" s="98"/>
-      <x:c r="Y73" s="5"/>
-      <x:c r="Z73" s="5"/>
-      <x:c r="AA73" s="5"/>
-      <x:c r="AB73" s="118"/>
-      <x:c r="AC73" s="119"/>
-      <x:c r="AD73" s="119"/>
+        <x:v>Открыт</x:v>
+      </x:c>
+      <x:c r="X73" s="98" t="str">
+        <x:v>Ещё 2 гола: полный выигрыш; 1: полупроигрыш; 0: проигрыш. 1 условная единица. Внешнее обогащение не применялось: нет конкретного уточнения, способного изменить отбор.</x:v>
+      </x:c>
+      <x:c r="Y73" s="5" t="str">
+        <x:v>Оптимальный</x:v>
+      </x:c>
+      <x:c r="Z73" s="5" t="str">
+        <x:v>20261014T171124-11168551</x:v>
+      </x:c>
+      <x:c r="AA73" s="5" t="str">
+        <x:v>Матч</x:v>
+      </x:c>
+      <x:c r="AB73" s="118" t="n">
+        <x:v>3.25</x:v>
+      </x:c>
+      <x:c r="AC73" s="119" t="str">
+        <x:v>14.10.2026 17:11:23</x:v>
+      </x:c>
+      <x:c r="AD73" s="119" t="str">
+        <x:v>14.10.2026 17:12:32</x:v>
+      </x:c>
       <x:c r="AE73" s="5" t="str">
         <x:f>IF(A73="","",IF(Z73="","Нет ID пары",IF(AND(COUNTIFS($Z$59:$Z$505,Z73,$Y$59:$Y$505,"Оптимальный",$W$59:$W$505,"Рассчитан")=1,COUNTIFS($Z$59:$Z$505,Z73,$Y$59:$Y$505,"Агрессивный",$W$59:$W$505,"Рассчитан")=1),"Да","Нет")))</x:f>
+        <x:v>Нет</x:v>
       </x:c>
       <x:c r="AF73" s="5"/>
-      <x:c r="AG73" s="5"/>
+      <x:c r="AG73" s="5" t="str">
+        <x:v>Два контура v2</x:v>
+      </x:c>
     </x:row>
     <x:row r="74">
-      <x:c r="A74" s="80"/>
-      <x:c r="B74" s="80"/>
-      <x:c r="C74" s="83"/>
-      <x:c r="D74" s="80"/>
-      <x:c r="E74" s="80"/>
-      <x:c r="F74" s="86"/>
-      <x:c r="G74" s="80"/>
-      <x:c r="H74" s="95"/>
-      <x:c r="I74" s="95"/>
-      <x:c r="J74" s="96"/>
-      <x:c r="K74" s="97"/>
-      <x:c r="L74" s="98"/>
-      <x:c r="M74" s="98"/>
-      <x:c r="N74" s="98"/>
-      <x:c r="O74" s="98"/>
-      <x:c r="P74" s="98"/>
-      <x:c r="Q74" s="80"/>
-      <x:c r="R74" s="80"/>
-      <x:c r="S74" s="80"/>
+      <x:c r="A74" s="80" t="n">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="B74" s="80" t="str">
+        <x:v>11168551</x:v>
+      </x:c>
+      <x:c r="C74" s="83" t="str">
+        <x:v>14.10.2026 17:11:23</x:v>
+      </x:c>
+      <x:c r="D74" s="80" t="str">
+        <x:v>Норвегия — 1-й дивизион</x:v>
+      </x:c>
+      <x:c r="E74" s="80" t="str">
+        <x:v>Стрёммен - Осане</x:v>
+      </x:c>
+      <x:c r="F74" s="86" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="G74" s="80" t="str">
+        <x:v>2:0</x:v>
+      </x:c>
+      <x:c r="H74" s="95" t="str">
+        <x:v>Высокий объём ударов при преимуществе хозяев; возможны голы через давление хозяев и попытки гостей отыграться.</x:v>
+      </x:c>
+      <x:c r="I74" s="95" t="str">
+        <x:v>ТБ 3.75 матча</x:v>
+      </x:c>
+      <x:c r="J74" s="96" t="n">
+        <x:v>2.075</x:v>
+      </x:c>
+      <x:c r="K74" s="97" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L74" s="98" t="str">
+        <x:v>Взрослый мужской. В створ 6:1; мимо 5:9; опасные атаки 50:35; угловые 7:3; xG отсутствует.</x:v>
+      </x:c>
+      <x:c r="M74" s="98" t="str">
+        <x:v>2893.5 с между срезами; минута 22 → 53; с перерывом; не окно 10–15 минут. Прирост в створ 5:1, мимо 4:3, угловые 5:1, опасные атаки 30:25.</x:v>
+      </x:c>
+      <x:c r="N74" s="98" t="str">
+        <x:v>21 удар, в створ 6:1, угловые 7:3. Хозяева способны создавать голы сами, гости отвечают объёмом ударов.</x:v>
+      </x:c>
+      <x:c r="O74" s="98" t="str">
+        <x:v>При 2:0 хозяева могут снижать темп; у гостей лишь 1 удар в створ. Нет xG и короткого интервала динамики.</x:v>
+      </x:c>
+      <x:c r="P74" s="98" t="str">
+        <x:v>Есть счёт, минута, статистика и активные линии; нет xG и динамики за 10–15 минут.</x:v>
+      </x:c>
+      <x:c r="Q74" s="80" t="str">
+        <x:v>ПОДХОДИТ В LIVE</x:v>
+      </x:c>
+      <x:c r="R74" s="80" t="str">
+        <x:v>Канон 14.10.2026; быстрый отбор + сохранение срезов</x:v>
+      </x:c>
+      <x:c r="S74" s="80" t="str">
+        <x:v>BetsAPI Events board + Bet365 full markets; run 38578271681</x:v>
+      </x:c>
       <x:c r="T74" s="80"/>
       <x:c r="U74" s="80"/>
       <x:c r="V74" s="89" t="str">
@@ -7717,40 +7870,96 @@
       </x:c>
       <x:c r="W74" s="80" t="str">
         <x:f>IF(A74="","",IF(U74="","Открыт",IF(ISNUMBER(V74),"Рассчитан","Проверить результат")))</x:f>
-      </x:c>
-      <x:c r="X74" s="98"/>
-      <x:c r="Y74" s="5"/>
-      <x:c r="Z74" s="5"/>
-      <x:c r="AA74" s="5"/>
-      <x:c r="AB74" s="118"/>
-      <x:c r="AC74" s="119"/>
-      <x:c r="AD74" s="119"/>
+        <x:v>Открыт</x:v>
+      </x:c>
+      <x:c r="X74" s="98" t="str">
+        <x:v>Ещё 3 гола: полный выигрыш; 2: полувыигрыш; 0–1: проигрыш. 1 условная единица. Внешнее обогащение не применялось: нет конкретного уточнения, способного изменить отбор.</x:v>
+      </x:c>
+      <x:c r="Y74" s="5" t="str">
+        <x:v>Агрессивный</x:v>
+      </x:c>
+      <x:c r="Z74" s="5" t="str">
+        <x:v>20261014T171124-11168551</x:v>
+      </x:c>
+      <x:c r="AA74" s="5" t="str">
+        <x:v>Матч</x:v>
+      </x:c>
+      <x:c r="AB74" s="118" t="n">
+        <x:v>3.75</x:v>
+      </x:c>
+      <x:c r="AC74" s="119" t="str">
+        <x:v>14.10.2026 17:11:23</x:v>
+      </x:c>
+      <x:c r="AD74" s="119" t="str">
+        <x:v>14.10.2026 17:12:32</x:v>
+      </x:c>
       <x:c r="AE74" s="5" t="str">
         <x:f>IF(A74="","",IF(Z74="","Нет ID пары",IF(AND(COUNTIFS($Z$59:$Z$505,Z74,$Y$59:$Y$505,"Оптимальный",$W$59:$W$505,"Рассчитан")=1,COUNTIFS($Z$59:$Z$505,Z74,$Y$59:$Y$505,"Агрессивный",$W$59:$W$505,"Рассчитан")=1),"Да","Нет")))</x:f>
+        <x:v>Нет</x:v>
       </x:c>
       <x:c r="AF74" s="5"/>
-      <x:c r="AG74" s="5"/>
+      <x:c r="AG74" s="5" t="str">
+        <x:v>Два контура v2</x:v>
+      </x:c>
     </x:row>
     <x:row r="75">
-      <x:c r="A75" s="80"/>
-      <x:c r="B75" s="80"/>
-      <x:c r="C75" s="83"/>
-      <x:c r="D75" s="80"/>
-      <x:c r="E75" s="80"/>
-      <x:c r="F75" s="86"/>
-      <x:c r="G75" s="80"/>
-      <x:c r="H75" s="95"/>
-      <x:c r="I75" s="95"/>
-      <x:c r="J75" s="96"/>
-      <x:c r="K75" s="97"/>
-      <x:c r="L75" s="98"/>
-      <x:c r="M75" s="98"/>
-      <x:c r="N75" s="98"/>
-      <x:c r="O75" s="98"/>
-      <x:c r="P75" s="98"/>
-      <x:c r="Q75" s="80"/>
-      <x:c r="R75" s="80"/>
-      <x:c r="S75" s="80"/>
+      <x:c r="A75" s="80" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="B75" s="80" t="str">
+        <x:v>13293139</x:v>
+      </x:c>
+      <x:c r="C75" s="83" t="str">
+        <x:v>14.10.2026 17:11:23</x:v>
+      </x:c>
+      <x:c r="D75" s="80" t="str">
+        <x:v>Египет — второй дивизион B</x:v>
+      </x:c>
+      <x:c r="E75" s="80" t="str">
+        <x:v>Каскада - Джи ФК</x:v>
+      </x:c>
+      <x:c r="F75" s="86" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="G75" s="80" t="str">
+        <x:v>0:2</x:v>
+      </x:c>
+      <x:c r="H75" s="95" t="str">
+        <x:v>Взаимная угроза и попытки хозяев вернуться в матч создают условия для следующих голов.</x:v>
+      </x:c>
+      <x:c r="I75" s="95" t="str">
+        <x:v>ТБ 3 матча</x:v>
+      </x:c>
+      <x:c r="J75" s="96" t="n">
+        <x:v>1.825</x:v>
+      </x:c>
+      <x:c r="K75" s="97" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L75" s="98" t="str">
+        <x:v>Взрослый мужской. В створ 3:5; мимо 7:4; опасные атаки 51:41; угловые 2:3; xG отсутствует.</x:v>
+      </x:c>
+      <x:c r="M75" s="98" t="str">
+        <x:v>2893.5 с между срезами; минута 39 → 55; с перерывом; не окно 10–15 минут. Прирост в створ 1:2, мимо 2:2, угловые 2:1, опасные атаки 19:13.</x:v>
+      </x:c>
+      <x:c r="N75" s="98" t="str">
+        <x:v>В створ 3:5, мимо 7:4, опасные атаки 51:41. Угроза с обеих сторон при необходимости хозяев отыгрываться.</x:v>
+      </x:c>
+      <x:c r="O75" s="98" t="str">
+        <x:v>Гости ведут 0:2 и могут перейти к удержанию. Нет xG и короткого интервала динамики.</x:v>
+      </x:c>
+      <x:c r="P75" s="98" t="str">
+        <x:v>Есть счёт, минута, статистика и активные линии; нет xG и динамики за 10–15 минут.</x:v>
+      </x:c>
+      <x:c r="Q75" s="80" t="str">
+        <x:v>ПОДХОДИТ В LIVE</x:v>
+      </x:c>
+      <x:c r="R75" s="80" t="str">
+        <x:v>Канон 14.10.2026; быстрый отбор + сохранение срезов</x:v>
+      </x:c>
+      <x:c r="S75" s="80" t="str">
+        <x:v>BetsAPI Events board + Bet365 full markets; run 38578271681</x:v>
+      </x:c>
       <x:c r="T75" s="80"/>
       <x:c r="U75" s="80"/>
       <x:c r="V75" s="89" t="str">
@@ -7758,40 +7967,96 @@
       </x:c>
       <x:c r="W75" s="80" t="str">
         <x:f>IF(A75="","",IF(U75="","Открыт",IF(ISNUMBER(V75),"Рассчитан","Проверить результат")))</x:f>
-      </x:c>
-      <x:c r="X75" s="98"/>
-      <x:c r="Y75" s="5"/>
-      <x:c r="Z75" s="5"/>
-      <x:c r="AA75" s="5"/>
-      <x:c r="AB75" s="118"/>
-      <x:c r="AC75" s="119"/>
-      <x:c r="AD75" s="119"/>
+        <x:v>Открыт</x:v>
+      </x:c>
+      <x:c r="X75" s="98" t="str">
+        <x:v>Ещё 2 гола: выигрыш; 1: возврат; 0: проигрыш. 1 условная единица. Внешнее обогащение не применялось: нет конкретного уточнения, способного изменить отбор.</x:v>
+      </x:c>
+      <x:c r="Y75" s="5" t="str">
+        <x:v>Оптимальный</x:v>
+      </x:c>
+      <x:c r="Z75" s="5" t="str">
+        <x:v>20261014T171124-13293139</x:v>
+      </x:c>
+      <x:c r="AA75" s="5" t="str">
+        <x:v>Матч</x:v>
+      </x:c>
+      <x:c r="AB75" s="118" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="AC75" s="119" t="str">
+        <x:v>14.10.2026 17:11:23</x:v>
+      </x:c>
+      <x:c r="AD75" s="119" t="str">
+        <x:v>14.10.2026 17:12:32</x:v>
+      </x:c>
       <x:c r="AE75" s="5" t="str">
         <x:f>IF(A75="","",IF(Z75="","Нет ID пары",IF(AND(COUNTIFS($Z$59:$Z$505,Z75,$Y$59:$Y$505,"Оптимальный",$W$59:$W$505,"Рассчитан")=1,COUNTIFS($Z$59:$Z$505,Z75,$Y$59:$Y$505,"Агрессивный",$W$59:$W$505,"Рассчитан")=1),"Да","Нет")))</x:f>
+        <x:v>Нет</x:v>
       </x:c>
       <x:c r="AF75" s="5"/>
-      <x:c r="AG75" s="5"/>
+      <x:c r="AG75" s="5" t="str">
+        <x:v>Два контура v2</x:v>
+      </x:c>
     </x:row>
     <x:row r="76">
-      <x:c r="A76" s="80"/>
-      <x:c r="B76" s="80"/>
-      <x:c r="C76" s="83"/>
-      <x:c r="D76" s="80"/>
-      <x:c r="E76" s="80"/>
-      <x:c r="F76" s="86"/>
-      <x:c r="G76" s="80"/>
-      <x:c r="H76" s="95"/>
-      <x:c r="I76" s="95"/>
-      <x:c r="J76" s="96"/>
-      <x:c r="K76" s="97"/>
-      <x:c r="L76" s="98"/>
-      <x:c r="M76" s="98"/>
-      <x:c r="N76" s="98"/>
-      <x:c r="O76" s="98"/>
-      <x:c r="P76" s="98"/>
-      <x:c r="Q76" s="80"/>
-      <x:c r="R76" s="80"/>
-      <x:c r="S76" s="80"/>
+      <x:c r="A76" s="80" t="n">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B76" s="80" t="str">
+        <x:v>13293139</x:v>
+      </x:c>
+      <x:c r="C76" s="83" t="str">
+        <x:v>14.10.2026 17:11:23</x:v>
+      </x:c>
+      <x:c r="D76" s="80" t="str">
+        <x:v>Египет — второй дивизион B</x:v>
+      </x:c>
+      <x:c r="E76" s="80" t="str">
+        <x:v>Каскада - Джи ФК</x:v>
+      </x:c>
+      <x:c r="F76" s="86" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="G76" s="80" t="str">
+        <x:v>0:2</x:v>
+      </x:c>
+      <x:c r="H76" s="95" t="str">
+        <x:v>Взаимная угроза и попытки хозяев вернуться в матч создают условия для следующих голов.</x:v>
+      </x:c>
+      <x:c r="I76" s="95" t="str">
+        <x:v>ТБ 3.5 матча</x:v>
+      </x:c>
+      <x:c r="J76" s="96" t="n">
+        <x:v>2.75</x:v>
+      </x:c>
+      <x:c r="K76" s="97" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L76" s="98" t="str">
+        <x:v>Взрослый мужской. В створ 3:5; мимо 7:4; опасные атаки 51:41; угловые 2:3; xG отсутствует.</x:v>
+      </x:c>
+      <x:c r="M76" s="98" t="str">
+        <x:v>2893.5 с между срезами; минута 39 → 55; с перерывом; не окно 10–15 минут. Прирост в створ 1:2, мимо 2:2, угловые 2:1, опасные атаки 19:13.</x:v>
+      </x:c>
+      <x:c r="N76" s="98" t="str">
+        <x:v>В створ 3:5, мимо 7:4, опасные атаки 51:41. Угроза с обеих сторон при необходимости хозяев отыгрываться.</x:v>
+      </x:c>
+      <x:c r="O76" s="98" t="str">
+        <x:v>Гости ведут 0:2 и могут перейти к удержанию. Нет xG и короткого интервала динамики.</x:v>
+      </x:c>
+      <x:c r="P76" s="98" t="str">
+        <x:v>Есть счёт, минута, статистика и активные линии; нет xG и динамики за 10–15 минут.</x:v>
+      </x:c>
+      <x:c r="Q76" s="80" t="str">
+        <x:v>ПОДХОДИТ В LIVE</x:v>
+      </x:c>
+      <x:c r="R76" s="80" t="str">
+        <x:v>Канон 14.10.2026; быстрый отбор + сохранение срезов</x:v>
+      </x:c>
+      <x:c r="S76" s="80" t="str">
+        <x:v>BetsAPI Events board + Bet365 full markets; run 38578271681</x:v>
+      </x:c>
       <x:c r="T76" s="80"/>
       <x:c r="U76" s="80"/>
       <x:c r="V76" s="89" t="str">
@@ -7799,40 +8064,96 @@
       </x:c>
       <x:c r="W76" s="80" t="str">
         <x:f>IF(A76="","",IF(U76="","Открыт",IF(ISNUMBER(V76),"Рассчитан","Проверить результат")))</x:f>
-      </x:c>
-      <x:c r="X76" s="98"/>
-      <x:c r="Y76" s="5"/>
-      <x:c r="Z76" s="5"/>
-      <x:c r="AA76" s="5"/>
-      <x:c r="AB76" s="118"/>
-      <x:c r="AC76" s="119"/>
-      <x:c r="AD76" s="119"/>
+        <x:v>Открыт</x:v>
+      </x:c>
+      <x:c r="X76" s="98" t="str">
+        <x:v>Ещё 2 гола: выигрыш; 0–1: проигрыш. 1 условная единица. Внешнее обогащение не применялось: нет конкретного уточнения, способного изменить отбор.</x:v>
+      </x:c>
+      <x:c r="Y76" s="5" t="str">
+        <x:v>Агрессивный</x:v>
+      </x:c>
+      <x:c r="Z76" s="5" t="str">
+        <x:v>20261014T171124-13293139</x:v>
+      </x:c>
+      <x:c r="AA76" s="5" t="str">
+        <x:v>Матч</x:v>
+      </x:c>
+      <x:c r="AB76" s="118" t="n">
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="AC76" s="119" t="str">
+        <x:v>14.10.2026 17:11:23</x:v>
+      </x:c>
+      <x:c r="AD76" s="119" t="str">
+        <x:v>14.10.2026 17:12:32</x:v>
+      </x:c>
       <x:c r="AE76" s="5" t="str">
         <x:f>IF(A76="","",IF(Z76="","Нет ID пары",IF(AND(COUNTIFS($Z$59:$Z$505,Z76,$Y$59:$Y$505,"Оптимальный",$W$59:$W$505,"Рассчитан")=1,COUNTIFS($Z$59:$Z$505,Z76,$Y$59:$Y$505,"Агрессивный",$W$59:$W$505,"Рассчитан")=1),"Да","Нет")))</x:f>
+        <x:v>Нет</x:v>
       </x:c>
       <x:c r="AF76" s="5"/>
-      <x:c r="AG76" s="5"/>
+      <x:c r="AG76" s="5" t="str">
+        <x:v>Два контура v2</x:v>
+      </x:c>
     </x:row>
     <x:row r="77">
-      <x:c r="A77" s="80"/>
-      <x:c r="B77" s="80"/>
-      <x:c r="C77" s="83"/>
-      <x:c r="D77" s="80"/>
-      <x:c r="E77" s="80"/>
-      <x:c r="F77" s="86"/>
-      <x:c r="G77" s="80"/>
-      <x:c r="H77" s="95"/>
-      <x:c r="I77" s="95"/>
-      <x:c r="J77" s="96"/>
-      <x:c r="K77" s="97"/>
-      <x:c r="L77" s="98"/>
-      <x:c r="M77" s="98"/>
-      <x:c r="N77" s="98"/>
-      <x:c r="O77" s="98"/>
-      <x:c r="P77" s="98"/>
-      <x:c r="Q77" s="80"/>
-      <x:c r="R77" s="80"/>
-      <x:c r="S77" s="80"/>
+      <x:c r="A77" s="80" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="B77" s="80" t="str">
+        <x:v>11560445</x:v>
+      </x:c>
+      <x:c r="C77" s="83" t="str">
+        <x:v>14.10.2026 17:11:23</x:v>
+      </x:c>
+      <x:c r="D77" s="80" t="str">
+        <x:v>Эстония — Мейстрилига</x:v>
+      </x:c>
+      <x:c r="E77" s="80" t="str">
+        <x:v>Нарва Транс - Курессааре</x:v>
+      </x:c>
+      <x:c r="F77" s="86" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="G77" s="80" t="str">
+        <x:v>0:0</x:v>
+      </x:c>
+      <x:c r="H77" s="95" t="str">
+        <x:v>Один или два гола во втором тайме при взаимной угрозе и равном счёте.</x:v>
+      </x:c>
+      <x:c r="I77" s="95" t="str">
+        <x:v>ТБ 1 матча</x:v>
+      </x:c>
+      <x:c r="J77" s="96" t="n">
+        <x:v>1.575</x:v>
+      </x:c>
+      <x:c r="K77" s="97" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L77" s="98" t="str">
+        <x:v>Взрослый мужской. В створ 2:4; мимо 0:2; опасные атаки 32:27; угловые 2:2; xG отсутствует.</x:v>
+      </x:c>
+      <x:c r="M77" s="98" t="str">
+        <x:v>2893.5 с между срезами; минута 21 → 53; с перерывом; не окно 10–15 минут. Прирост в створ 1:2, мимо 0:0, угловые 1:1, опасные атаки 22:15.</x:v>
+      </x:c>
+      <x:c r="N77" s="98" t="str">
+        <x:v>В створ 2:4, опасные атаки 32:27. Угроза обеих сторон сочетается с низкой линией.</x:v>
+      </x:c>
+      <x:c r="O77" s="98" t="str">
+        <x:v>Всего 8 ударов, общий темп умеренный. Нет xG и короткого интервала динамики.</x:v>
+      </x:c>
+      <x:c r="P77" s="98" t="str">
+        <x:v>Есть счёт, минута, статистика и активные линии; нет xG и динамики за 10–15 минут.</x:v>
+      </x:c>
+      <x:c r="Q77" s="80" t="str">
+        <x:v>ПОДХОДИТ В LIVE</x:v>
+      </x:c>
+      <x:c r="R77" s="80" t="str">
+        <x:v>Канон 14.10.2026; быстрый отбор + сохранение срезов</x:v>
+      </x:c>
+      <x:c r="S77" s="80" t="str">
+        <x:v>BetsAPI Events board + Bet365 full markets; run 38578271681</x:v>
+      </x:c>
       <x:c r="T77" s="80"/>
       <x:c r="U77" s="80"/>
       <x:c r="V77" s="89" t="str">
@@ -7840,40 +8161,96 @@
       </x:c>
       <x:c r="W77" s="80" t="str">
         <x:f>IF(A77="","",IF(U77="","Открыт",IF(ISNUMBER(V77),"Рассчитан","Проверить результат")))</x:f>
-      </x:c>
-      <x:c r="X77" s="98"/>
-      <x:c r="Y77" s="5"/>
-      <x:c r="Z77" s="5"/>
-      <x:c r="AA77" s="5"/>
-      <x:c r="AB77" s="118"/>
-      <x:c r="AC77" s="119"/>
-      <x:c r="AD77" s="119"/>
+        <x:v>Открыт</x:v>
+      </x:c>
+      <x:c r="X77" s="98" t="str">
+        <x:v>Ещё 2 гола: выигрыш; 1: возврат; 0: проигрыш. 1 условная единица. Внешнее обогащение не применялось: нет конкретного уточнения, способного изменить отбор.</x:v>
+      </x:c>
+      <x:c r="Y77" s="5" t="str">
+        <x:v>Оптимальный</x:v>
+      </x:c>
+      <x:c r="Z77" s="5" t="str">
+        <x:v>20261014T171124-11560445</x:v>
+      </x:c>
+      <x:c r="AA77" s="5" t="str">
+        <x:v>Матч</x:v>
+      </x:c>
+      <x:c r="AB77" s="118" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AC77" s="119" t="str">
+        <x:v>14.10.2026 17:11:23</x:v>
+      </x:c>
+      <x:c r="AD77" s="119" t="str">
+        <x:v>14.10.2026 17:12:32</x:v>
+      </x:c>
       <x:c r="AE77" s="5" t="str">
         <x:f>IF(A77="","",IF(Z77="","Нет ID пары",IF(AND(COUNTIFS($Z$59:$Z$505,Z77,$Y$59:$Y$505,"Оптимальный",$W$59:$W$505,"Рассчитан")=1,COUNTIFS($Z$59:$Z$505,Z77,$Y$59:$Y$505,"Агрессивный",$W$59:$W$505,"Рассчитан")=1),"Да","Нет")))</x:f>
+        <x:v>Нет</x:v>
       </x:c>
       <x:c r="AF77" s="5"/>
-      <x:c r="AG77" s="5"/>
+      <x:c r="AG77" s="5" t="str">
+        <x:v>Два контура v2</x:v>
+      </x:c>
     </x:row>
     <x:row r="78">
-      <x:c r="A78" s="80"/>
-      <x:c r="B78" s="80"/>
-      <x:c r="C78" s="83"/>
-      <x:c r="D78" s="80"/>
-      <x:c r="E78" s="80"/>
-      <x:c r="F78" s="86"/>
-      <x:c r="G78" s="80"/>
-      <x:c r="H78" s="95"/>
-      <x:c r="I78" s="95"/>
-      <x:c r="J78" s="96"/>
-      <x:c r="K78" s="97"/>
-      <x:c r="L78" s="98"/>
-      <x:c r="M78" s="98"/>
-      <x:c r="N78" s="98"/>
-      <x:c r="O78" s="98"/>
-      <x:c r="P78" s="98"/>
-      <x:c r="Q78" s="80"/>
-      <x:c r="R78" s="80"/>
-      <x:c r="S78" s="80"/>
+      <x:c r="A78" s="80" t="n">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="B78" s="80" t="str">
+        <x:v>11560445</x:v>
+      </x:c>
+      <x:c r="C78" s="83" t="str">
+        <x:v>14.10.2026 17:11:23</x:v>
+      </x:c>
+      <x:c r="D78" s="80" t="str">
+        <x:v>Эстония — Мейстрилига</x:v>
+      </x:c>
+      <x:c r="E78" s="80" t="str">
+        <x:v>Нарва Транс - Курессааре</x:v>
+      </x:c>
+      <x:c r="F78" s="86" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="G78" s="80" t="str">
+        <x:v>0:0</x:v>
+      </x:c>
+      <x:c r="H78" s="95" t="str">
+        <x:v>Один или два гола во втором тайме при взаимной угрозе и равном счёте.</x:v>
+      </x:c>
+      <x:c r="I78" s="95" t="str">
+        <x:v>ТБ 1.25 матча</x:v>
+      </x:c>
+      <x:c r="J78" s="96" t="n">
+        <x:v>1.975</x:v>
+      </x:c>
+      <x:c r="K78" s="97" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L78" s="98" t="str">
+        <x:v>Взрослый мужской. В створ 2:4; мимо 0:2; опасные атаки 32:27; угловые 2:2; xG отсутствует.</x:v>
+      </x:c>
+      <x:c r="M78" s="98" t="str">
+        <x:v>2893.5 с между срезами; минута 21 → 53; с перерывом; не окно 10–15 минут. Прирост в створ 1:2, мимо 0:0, угловые 1:1, опасные атаки 22:15.</x:v>
+      </x:c>
+      <x:c r="N78" s="98" t="str">
+        <x:v>В створ 2:4, опасные атаки 32:27. Угроза обеих сторон сочетается с низкой линией.</x:v>
+      </x:c>
+      <x:c r="O78" s="98" t="str">
+        <x:v>Всего 8 ударов, общий темп умеренный. Нет xG и короткого интервала динамики.</x:v>
+      </x:c>
+      <x:c r="P78" s="98" t="str">
+        <x:v>Есть счёт, минута, статистика и активные линии; нет xG и динамики за 10–15 минут.</x:v>
+      </x:c>
+      <x:c r="Q78" s="80" t="str">
+        <x:v>ПОДХОДИТ В LIVE</x:v>
+      </x:c>
+      <x:c r="R78" s="80" t="str">
+        <x:v>Канон 14.10.2026; быстрый отбор + сохранение срезов</x:v>
+      </x:c>
+      <x:c r="S78" s="80" t="str">
+        <x:v>BetsAPI Events board + Bet365 full markets; run 38578271681</x:v>
+      </x:c>
       <x:c r="T78" s="80"/>
       <x:c r="U78" s="80"/>
       <x:c r="V78" s="89" t="str">
@@ -7881,19 +8258,37 @@
       </x:c>
       <x:c r="W78" s="80" t="str">
         <x:f>IF(A78="","",IF(U78="","Открыт",IF(ISNUMBER(V78),"Рассчитан","Проверить результат")))</x:f>
-      </x:c>
-      <x:c r="X78" s="98"/>
-      <x:c r="Y78" s="5"/>
-      <x:c r="Z78" s="5"/>
-      <x:c r="AA78" s="5"/>
-      <x:c r="AB78" s="118"/>
-      <x:c r="AC78" s="119"/>
-      <x:c r="AD78" s="119"/>
+        <x:v>Открыт</x:v>
+      </x:c>
+      <x:c r="X78" s="98" t="str">
+        <x:v>Ещё 2 гола: выигрыш; 1: полупроигрыш; 0: проигрыш. 1 условная единица. Внешнее обогащение не применялось: нет конкретного уточнения, способного изменить отбор.</x:v>
+      </x:c>
+      <x:c r="Y78" s="5" t="str">
+        <x:v>Агрессивный</x:v>
+      </x:c>
+      <x:c r="Z78" s="5" t="str">
+        <x:v>20261014T171124-11560445</x:v>
+      </x:c>
+      <x:c r="AA78" s="5" t="str">
+        <x:v>Матч</x:v>
+      </x:c>
+      <x:c r="AB78" s="118" t="n">
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="AC78" s="119" t="str">
+        <x:v>14.10.2026 17:11:23</x:v>
+      </x:c>
+      <x:c r="AD78" s="119" t="str">
+        <x:v>14.10.2026 17:12:32</x:v>
+      </x:c>
       <x:c r="AE78" s="5" t="str">
         <x:f>IF(A78="","",IF(Z78="","Нет ID пары",IF(AND(COUNTIFS($Z$59:$Z$505,Z78,$Y$59:$Y$505,"Оптимальный",$W$59:$W$505,"Рассчитан")=1,COUNTIFS($Z$59:$Z$505,Z78,$Y$59:$Y$505,"Агрессивный",$W$59:$W$505,"Рассчитан")=1),"Да","Нет")))</x:f>
+        <x:v>Нет</x:v>
       </x:c>
       <x:c r="AF78" s="5"/>
-      <x:c r="AG78" s="5"/>
+      <x:c r="AG78" s="5" t="str">
+        <x:v>Два контура v2</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="80"/>

</xml_diff>